<commit_message>
half comments done for k-copy
</commit_message>
<xml_diff>
--- a/comments.xlsx
+++ b/comments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webbd\Documents\phd\Scratch\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F81A3FD-CB71-4606-AF8D-35F21A39909F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BB6311-ECBD-47F3-B84E-95713AAFBAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>Chapter</t>
   </si>
@@ -85,19 +85,102 @@
   </si>
   <si>
     <t>SS</t>
+  </si>
+  <si>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t>k-copy:</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>1. adding more motivation at the start, and more explicitly describing what was new</t>
+  </si>
+  <si>
+    <t>2. Include the discussion we had on fitting a line to the early part of the decay? I know it's partially in the fisher information discussion but maybe worth being explicit?</t>
+  </si>
+  <si>
+    <t>3. Add the time correlation data</t>
+  </si>
+  <si>
+    <t>1) consider adding an attention grabber at the beginning of the chapter -- I think the classical repetition code could be a simple way to communicate the problem of correlated errors</t>
+  </si>
+  <si>
+    <t>2) the introductory paragraph to each section is currently just stating the contents of the section, I think adding a motivating statement building on the previous section would tie the story together</t>
+  </si>
+  <si>
+    <t>3) I would not attempt to do an exhaustive literature review; I think including correlated and sym RB and then pointing out why our method is different is sufficient</t>
+  </si>
+  <si>
+    <t>4) Having thought more about the parity measurements, I think I prefer to cast the measurement as being one of two-qubit correlations, rather than focussing on having an entangled state component. (see comment on page 25 for details)</t>
+  </si>
+  <si>
+    <t>5) In terms of formatting</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - ensure consistency in subscript case (whether to use \rm or not)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - ensure operators like diag and tr have consistent case</t>
+  </si>
+  <si>
+    <t>Conform all spin to $\downarrow,\uparrow$ rather than 0 and 1.</t>
+  </si>
+  <si>
+    <t>Conform (a), (b), \S , Fig, chapter references</t>
+  </si>
+  <si>
+    <t>Conform dashed and solid line for model vs fit</t>
+  </si>
+  <si>
+    <t>Conform all figure color schemes</t>
+  </si>
+  <si>
+    <t>General:</t>
+  </si>
+  <si>
+    <t>Conform all figure axis units to brackets</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1D1C1D"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF928374"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -138,11 +221,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,14 +554,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592C688F-CDAE-448C-B0E7-79FA2C7BB64E}">
-  <dimension ref="C4:L11"/>
+  <dimension ref="C4:T37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="9.140625" style="6"/>
+    <col min="19" max="19" width="46.85546875" style="6" customWidth="1"/>
+    <col min="20" max="20" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>0</v>
       </c>
@@ -493,7 +601,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>1</v>
       </c>
@@ -503,7 +611,7 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C6">
         <v>2</v>
       </c>
@@ -511,10 +619,10 @@
         <v>2</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="G6" s="5"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C7">
         <v>3</v>
       </c>
@@ -523,8 +631,9 @@
       </c>
       <c r="E7" s="3"/>
       <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>4</v>
       </c>
@@ -532,9 +641,9 @@
         <v>4</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>5</v>
       </c>
@@ -544,19 +653,19 @@
       <c r="E9" s="3"/>
       <c r="G9" s="3"/>
     </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C10">
         <v>6</v>
       </c>
       <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="3"/>
       <c r="G10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
     </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>7</v>
       </c>
@@ -566,7 +675,124 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
+    <row r="12" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="Q13" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="3:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="S14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="T14"/>
+    </row>
+    <row r="15" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="S15" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="T15"/>
+    </row>
+    <row r="16" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="S16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="T16"/>
+    </row>
+    <row r="17" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S17" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="T17"/>
+    </row>
+    <row r="18" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S18" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="T18"/>
+    </row>
+    <row r="19" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="T19"/>
+    </row>
+    <row r="20" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="T20"/>
+    </row>
+    <row r="21" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S21" s="9"/>
+      <c r="T21"/>
+    </row>
+    <row r="22" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S22" s="9"/>
+      <c r="T22"/>
+    </row>
+    <row r="26" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="Q26" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="17:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="R27" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="17:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="S28" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S29" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="17:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="R31" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="S31" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="17:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="S32" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="19:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="S33" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="19:19" ht="90" x14ac:dyDescent="0.25">
+      <c r="S34" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S35" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="19:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="S36" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="19:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="S37" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
comments done for k-copy chapter
</commit_message>
<xml_diff>
--- a/comments.xlsx
+++ b/comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webbd\Documents\phd\Scratch\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BB6311-ECBD-47F3-B84E-95713AAFBAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D9F30B-8497-40EB-AAD7-02DFDE1A1563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>Chapter</t>
   </si>
@@ -96,36 +96,9 @@
     <t>RS</t>
   </si>
   <si>
-    <t>1. adding more motivation at the start, and more explicitly describing what was new</t>
-  </si>
-  <si>
-    <t>2. Include the discussion we had on fitting a line to the early part of the decay? I know it's partially in the fisher information discussion but maybe worth being explicit?</t>
-  </si>
-  <si>
     <t>3. Add the time correlation data</t>
   </si>
   <si>
-    <t>1) consider adding an attention grabber at the beginning of the chapter -- I think the classical repetition code could be a simple way to communicate the problem of correlated errors</t>
-  </si>
-  <si>
-    <t>2) the introductory paragraph to each section is currently just stating the contents of the section, I think adding a motivating statement building on the previous section would tie the story together</t>
-  </si>
-  <si>
-    <t>3) I would not attempt to do an exhaustive literature review; I think including correlated and sym RB and then pointing out why our method is different is sufficient</t>
-  </si>
-  <si>
-    <t>4) Having thought more about the parity measurements, I think I prefer to cast the measurement as being one of two-qubit correlations, rather than focussing on having an entangled state component. (see comment on page 25 for details)</t>
-  </si>
-  <si>
-    <t>5) In terms of formatting</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - ensure consistency in subscript case (whether to use \rm or not)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - ensure operators like diag and tr have consistent case</t>
-  </si>
-  <si>
     <t>Conform all spin to $\downarrow,\uparrow$ rather than 0 and 1.</t>
   </si>
   <si>
@@ -142,13 +115,34 @@
   </si>
   <si>
     <t>Conform all figure axis units to brackets</t>
+  </si>
+  <si>
+    <t>Quantify the gain due to the EM on the &lt;Z_pur&gt; by quoting something like epsilon_pur and compare it to epsilon_l, epsilon_r and the theoretical expected gain</t>
+  </si>
+  <si>
+    <t>Hybrid+QEM:</t>
+  </si>
+  <si>
+    <t>Update refs if published</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) put this work into slightly better context in terms of what others have done, especially with regards to VD i.e. what is actually new here. </t>
+  </si>
+  <si>
+    <t>2) Needs summary/conclusion that unifies both parts of the chapter</t>
+  </si>
+  <si>
+    <t>overall the writing is maybe slightly less precise than in the k-copy chapter</t>
+  </si>
+  <si>
+    <t>Justify why 1.1 and 1.2 are in one chapter. Potentially you could resolve this by making the virtual distillation on hybrid systems a standalone section 1.3 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +174,12 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -221,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -239,6 +239,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592C688F-CDAE-448C-B0E7-79FA2C7BB64E}">
-  <dimension ref="C4:T37"/>
+  <dimension ref="C4:T36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
@@ -567,7 +576,8 @@
     <col min="10" max="10" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="9.140625" style="6"/>
+    <col min="17" max="17" width="14.140625" style="6" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" style="6"/>
     <col min="19" max="19" width="46.85546875" style="6" customWidth="1"/>
     <col min="20" max="20" width="9.140625" style="6"/>
   </cols>
@@ -647,7 +657,7 @@
       <c r="C9">
         <v>5</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="3"/>
@@ -683,40 +693,43 @@
     </row>
     <row r="13" spans="3:20" x14ac:dyDescent="0.25">
       <c r="Q13" s="6" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="3:20" ht="30" x14ac:dyDescent="0.25">
       <c r="S14" s="8" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="T14"/>
     </row>
     <row r="15" spans="3:20" x14ac:dyDescent="0.25">
       <c r="S15" s="8" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="T15"/>
     </row>
     <row r="16" spans="3:20" x14ac:dyDescent="0.25">
       <c r="S16" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="T16"/>
     </row>
     <row r="17" spans="17:20" x14ac:dyDescent="0.25">
       <c r="S17" s="8" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="T17"/>
     </row>
     <row r="18" spans="17:20" x14ac:dyDescent="0.25">
       <c r="S18" s="8" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="T18"/>
     </row>
     <row r="19" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S19" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="T19"/>
     </row>
     <row r="20" spans="17:20" x14ac:dyDescent="0.25">
@@ -735,7 +748,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="17:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="17:20" x14ac:dyDescent="0.25">
       <c r="R27" s="6" t="s">
         <v>18</v>
       </c>
@@ -743,52 +756,46 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="17:20" ht="60" x14ac:dyDescent="0.25">
-      <c r="S28" s="7" t="s">
-        <v>20</v>
-      </c>
+    <row r="28" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S28" s="7"/>
     </row>
     <row r="29" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S29" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="31" spans="17:20" ht="60" x14ac:dyDescent="0.25">
-      <c r="R31" s="6" t="s">
+      <c r="Q29" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="17:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="R30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S30" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="17:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="S31" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="18:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="R33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="S31" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="17:20" ht="60" x14ac:dyDescent="0.25">
-      <c r="S32" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="19:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="S33" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="19:19" ht="90" x14ac:dyDescent="0.25">
-      <c r="S34" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S35" s="6" t="s">
+      <c r="S33" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="18:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="R35" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="S35" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="18:19" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="S36" s="12" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="19:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="S36" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="19:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="S37" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
half comments done for chapter 6
</commit_message>
<xml_diff>
--- a/comments.xlsx
+++ b/comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webbd\Documents\phd\Scratch\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D9F30B-8497-40EB-AAD7-02DFDE1A1563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C28D78-0E7C-4109-8ECD-B5C7FB2C74CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>Chapter</t>
   </si>
@@ -136,6 +136,18 @@
   </si>
   <si>
     <t>Justify why 1.1 and 1.2 are in one chapter. Potentially you could resolve this by making the virtual distillation on hybrid systems a standalone section 1.3 </t>
+  </si>
+  <si>
+    <t>Spell check all</t>
+  </si>
+  <si>
+    <t>Remove align env eqn numbers</t>
+  </si>
+  <si>
+    <t>Capitalise all Figure, Table, Appendix</t>
+  </si>
+  <si>
+    <t>add hrefs to references</t>
   </si>
 </sst>
 </file>
@@ -165,13 +177,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF928374"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -181,6 +186,12 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF928374"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -234,20 +245,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -563,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592C688F-CDAE-448C-B0E7-79FA2C7BB64E}">
-  <dimension ref="C4:T36"/>
+  <dimension ref="C4:T37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
@@ -733,68 +744,80 @@
       <c r="T19"/>
     </row>
     <row r="20" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S20" s="6" t="s">
+        <v>33</v>
+      </c>
       <c r="T20"/>
     </row>
     <row r="21" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S21" s="9"/>
+      <c r="S21" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="T21"/>
     </row>
     <row r="22" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S22" s="9"/>
+      <c r="S22" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="T22"/>
     </row>
-    <row r="26" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="Q26" s="6" t="s">
+    <row r="23" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="S23" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="Q27" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="R27" s="6" t="s">
+    <row r="28" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="R28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="S27" s="7" t="s">
+      <c r="S28" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S28" s="7"/>
-    </row>
     <row r="29" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="Q29" s="6" t="s">
+      <c r="S29" s="7"/>
+    </row>
+    <row r="30" spans="17:20" x14ac:dyDescent="0.25">
+      <c r="Q30" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="17:20" ht="45" x14ac:dyDescent="0.25">
-      <c r="R30" s="6" t="s">
+    <row r="31" spans="17:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="R31" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="S30" s="6" t="s">
+      <c r="S31" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="17:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="S31" s="6" t="s">
+    <row r="32" spans="17:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="S32" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="18:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="R33" s="6" t="s">
+    <row r="34" spans="18:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="R34" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="S33" s="10" t="s">
+      <c r="S34" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="18:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="R35" s="6" t="s">
+    <row r="36" spans="18:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="R36" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="S35" s="11" t="s">
+      <c r="S36" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="18:19" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="S36" s="12" t="s">
+    <row r="37" spans="18:19" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="S37" s="11" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
initial comments for chapter 3 and 4
</commit_message>
<xml_diff>
--- a/comments.xlsx
+++ b/comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webbd\Documents\phd\Scratch\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C28D78-0E7C-4109-8ECD-B5C7FB2C74CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF72202D-3016-4B03-8EF0-0F28DE30362F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
   </bookViews>
@@ -232,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -259,6 +259,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -756,7 +759,7 @@
       <c r="T21"/>
     </row>
     <row r="22" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S22" s="6" t="s">
+      <c r="S22" s="13" t="s">
         <v>35</v>
       </c>
       <c r="T22"/>

</xml_diff>

<commit_message>
all done but acknowledgements
</commit_message>
<xml_diff>
--- a/comments.xlsx
+++ b/comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webbd\Documents\phd\Scratch\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D29550-4BC8-4B7A-9B1C-A0256A39E986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4D9063-A342-48D7-9145-5139F3E9BBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{B0BE7E65-119E-4DBE-B1D0-25C3DFBD4425}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Chapter</t>
   </si>
@@ -90,15 +90,6 @@
     <t>Abstract</t>
   </si>
   <si>
-    <t>k-copy:</t>
-  </si>
-  <si>
-    <t>RS</t>
-  </si>
-  <si>
-    <t>3. Add the time correlation data</t>
-  </si>
-  <si>
     <t>Conform all spin to $\downarrow,\uparrow$ rather than 0 and 1.</t>
   </si>
   <si>
@@ -117,12 +108,6 @@
     <t>Conform all figure axis units to brackets</t>
   </si>
   <si>
-    <t>Hybrid+QEM:</t>
-  </si>
-  <si>
-    <t>2) Needs summary/conclusion that unifies both parts of the chapter</t>
-  </si>
-  <si>
     <t>Spell check all</t>
   </si>
   <si>
@@ -133,9 +118,6 @@
   </si>
   <si>
     <t>Capitalise all Figure, Table, Appendix, Chapter</t>
-  </si>
-  <si>
-    <t>I think my most major comment would be that I didn't see a mention of the reason the motion is used for entanglement,</t>
   </si>
   <si>
     <t>Update refs if published. I would hand off the .bib file to an AI and tell it to make sure all the references have authors, titles, journal (with standard and consistent abbreviations), volume, page number, and year, and the render in the tex file includes only this information</t>
@@ -145,7 +127,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,8 +166,15 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -195,12 +184,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -223,20 +206,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -247,14 +225,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,10 +564,10 @@
     <col min="10" max="10" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" style="5" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="5"/>
-    <col min="19" max="19" width="46.85546875" style="5" customWidth="1"/>
-    <col min="20" max="20" width="9.140625" style="5"/>
+    <col min="17" max="17" width="14.140625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" style="3"/>
+    <col min="19" max="19" width="46.85546875" style="3" customWidth="1"/>
+    <col min="20" max="20" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="4" spans="3:20" x14ac:dyDescent="0.25">
@@ -624,19 +606,19 @@
       <c r="D5" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="2"/>
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C6">
         <v>2</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="13"/>
+      <c r="E6" s="10"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
     </row>
     <row r="7" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C7">
@@ -645,9 +627,9 @@
       <c r="D7" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="E7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
     </row>
     <row r="8" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C8">
@@ -656,30 +638,30 @@
       <c r="D8" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="J8" s="3"/>
+      <c r="E8" s="10"/>
+      <c r="J8" s="2"/>
     </row>
     <row r="9" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>5</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C10">
         <v>6</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+      <c r="E10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
     </row>
     <row r="11" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C11">
@@ -688,132 +670,96 @@
       <c r="D11" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="3"/>
+      <c r="E11" s="2"/>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="3:20" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="2"/>
+      <c r="E12" s="13"/>
     </row>
     <row r="13" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="Q13" s="5" t="s">
+      <c r="Q13" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="3:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="S14" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="T14"/>
+    </row>
+    <row r="15" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="S15" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="T15"/>
+    </row>
+    <row r="16" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="S16" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="T16"/>
+    </row>
+    <row r="17" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S17" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="T17"/>
+    </row>
+    <row r="18" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S18" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="T18"/>
+    </row>
+    <row r="19" spans="19:20" ht="90" x14ac:dyDescent="0.25">
+      <c r="S19" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19"/>
+    </row>
+    <row r="20" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S20" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="T20"/>
+    </row>
+    <row r="21" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S21" s="11" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="3:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="S14" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="T14"/>
-    </row>
-    <row r="15" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="S15" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="T15"/>
-    </row>
-    <row r="16" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="S16" s="7" t="s">
+      <c r="T21"/>
+    </row>
+    <row r="22" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S22" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="T22"/>
+    </row>
+    <row r="23" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S23" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="T16"/>
-    </row>
-    <row r="17" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S17" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="T17"/>
-    </row>
-    <row r="18" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="T18"/>
-    </row>
-    <row r="19" spans="17:20" ht="90" x14ac:dyDescent="0.25">
-      <c r="S19" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="T19"/>
-    </row>
-    <row r="20" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S20" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="T20"/>
-    </row>
-    <row r="21" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S21" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="T21"/>
-    </row>
-    <row r="22" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S22" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="T22"/>
-    </row>
-    <row r="23" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S23" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="Q27" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="R28" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="S28" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="29" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="S29" s="6"/>
-    </row>
-    <row r="30" spans="17:20" x14ac:dyDescent="0.25">
-      <c r="Q30" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="17:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="R31" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="S31" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33" spans="17:19" x14ac:dyDescent="0.25">
-      <c r="Q33" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="17:19" x14ac:dyDescent="0.25">
-      <c r="S34" s="8"/>
-    </row>
-    <row r="35" spans="17:19" x14ac:dyDescent="0.25">
-      <c r="Q35" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="R35" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="S35" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="17:19" x14ac:dyDescent="0.25">
-      <c r="S36" s="9"/>
-    </row>
-    <row r="37" spans="17:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="S37" s="10"/>
+    </row>
+    <row r="28" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S28" s="4"/>
+    </row>
+    <row r="29" spans="19:20" x14ac:dyDescent="0.25">
+      <c r="S29" s="4"/>
+    </row>
+    <row r="34" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S34" s="5"/>
+    </row>
+    <row r="35" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S35"/>
+    </row>
+    <row r="36" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S36" s="6"/>
+    </row>
+    <row r="37" spans="19:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S37" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>